<commit_message>
Update project documentation and team task report #2
</commit_message>
<xml_diff>
--- a/docs/Task_Group_2.xlsx
+++ b/docs/Task_Group_2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Meterials\FPT\4. SUM26\PRJ301\PRJ301_SE2039_Group_2\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844ED6F0-9DCF-4EB4-A401-7B9202A040E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F418FDD6-4A76-4DA9-8AE0-2A680313A0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -317,7 +317,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -354,36 +354,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -396,16 +398,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -732,47 +731,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="32"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="15"/>
+      <c r="B3" s="32"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="15"/>
+      <c r="B4" s="32"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
       <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -788,10 +787,10 @@
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="23"/>
+      <c r="D8" s="25"/>
       <c r="E8" s="1" t="s">
         <v>4</v>
       </c>
@@ -803,14 +802,14 @@
       <c r="A9" s="4">
         <v>1</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="26" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="27"/>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="15" t="s">
         <v>7</v>
       </c>
       <c r="F9" s="12" t="s">
@@ -821,14 +820,14 @@
       <c r="A10" s="4">
         <v>2</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="14" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="26" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="27"/>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="15" t="s">
         <v>10</v>
       </c>
       <c r="F10" s="12" t="s">
@@ -839,14 +838,14 @@
       <c r="A11" s="4">
         <v>3</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="26" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="27"/>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="15" t="s">
         <v>12</v>
       </c>
       <c r="F11" s="12" t="s">
@@ -872,43 +871,42 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="31"/>
-      <c r="C13" s="30"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="7"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="str">
+      <c r="A14" s="31" t="str">
         <f>HYPERLINK(
-"https://github.com/phanthanhhung03/AutoWashPro-PRJ301-2.git",
-"https://github.com/phanthanhhung03/AutoWashPro-PRJ301-2.git"
+"https://github.com/phanthanhhung03/PRJ301_SE2039_Group_2.git",
+"https://github.com/phanthanhhung03/PRJ301_SE2039_Group_2.git"
 )</f>
-        <v>https://github.com/phanthanhhung03/AutoWashPro-PRJ301-2.git</v>
-      </c>
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="19"/>
+        <v>https://github.com/phanthanhhung03/PRJ301_SE2039_Group_2.git</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="16"/>
     </row>
     <row r="15" spans="1:6" s="9" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="24"/>
-      <c r="E15" s="20" t="s">
+      <c r="D15" s="17"/>
+      <c r="E15" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="20"/>
+      <c r="F15" s="23"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B16" s="21"/>
+      <c r="B16" s="20"/>
       <c r="C16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="25"/>
       <c r="E16" s="13" t="s">
         <v>15</v>
       </c>
@@ -917,14 +915,13 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="32"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="25"/>
       <c r="E17" s="13" t="s">
         <v>16</v>
       </c>
@@ -933,14 +930,13 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="32"/>
+      <c r="B18" s="19"/>
       <c r="C18" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="25"/>
       <c r="E18" s="13" t="s">
         <v>17</v>
       </c>
@@ -949,14 +945,13 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="32" t="s">
+      <c r="A19" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="32"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="25"/>
       <c r="E19" s="13" t="s">
         <v>18</v>
       </c>
@@ -965,10 +960,10 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="32"/>
+      <c r="B20" s="19"/>
       <c r="C20" s="2" t="s">
         <v>27</v>
       </c>

</xml_diff>